<commit_message>
Update taxonomy v0.2 with 8 gap fills: hallucination (general), crisis/self-harm, bias/discrimination (2), privacy/data exposure, jailbreak/safety bypass, misinformation amplification, shadow AI
Dee identified drift-heavy bias in taxonomy. Added non-drift failure categories from AIID analysis (18.5% discrimination, 12.8% misinformation, 7.6% privacy), OWASP LLM Top 10, and Perplexity Council findings. Corrected Amber role context (lab staff, not civilization agent). Total: 52 behaviors across 5 PRISM pillars.
</commit_message>
<xml_diff>
--- a/research/AUDACION_CITIZEN_OBSERVATION_TAXONOMY_v0.2.xlsx
+++ b/research/AUDACION_CITIZEN_OBSERVATION_TAXONOMY_v0.2.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +52,20 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -110,6 +122,16 @@
         <fgColor rgb="00D7BDE2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00922B21"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1948A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -137,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -171,6 +193,13 @@
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1599,8 +1628,280 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>GAP FILLS: Categories missing from v0.2 identified through AIID analysis and Dee's review</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>GAP FILL</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr"/>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>General Hallucination</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>OBS-P15</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>AI told me something plain wrong</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>Added: broadest hallucination category. Distinct from fabricated citation (P-03) and false certainty (P-09).</t>
+        </is>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>AIID GMF: Generalization Failure 44.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>GAP FILL</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr"/>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>Crisis/Self-Harm Context</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>OBS-P16</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>AI gave dangerous advice in crisis</t>
+        </is>
+      </c>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>Added: CRITICAL. AIID accelerating category. Amber processes this data for the lab.</t>
+        </is>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
+        <is>
+          <t>AIID: Character.AI, Gemini, Grok incidents</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>GAP FILL</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr"/>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Bias / Discriminatory Treatment</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>OBS-I10</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>AI treated me differently because of identity</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>Added: AIID 18.5% of incidents. Distinct from persona-dependent (OBS-I08).</t>
+        </is>
+      </c>
+      <c r="G41" s="14" t="inlineStr">
+        <is>
+          <t>AIID Harm: race 34.8%, sex 9.6%, religion 7.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>GAP FILL</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr"/>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>Biased/Toxic Output</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>OBS-I11</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>AI output was biased, stereotyping, offensive</t>
+        </is>
+      </c>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>Added: content-level bias. May be unintentional.</t>
+        </is>
+      </c>
+      <c r="G42" s="14" t="inlineStr">
+        <is>
+          <t>AIID GMF: Distributional Bias 6.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>GAP FILL</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr"/>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Privacy / Data Exposure</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>OBS-S10</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>AI revealed information it shouldn't have</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr">
+        <is>
+          <t>Added: OWASP LLM02. System prompt leakage, PII, training data.</t>
+        </is>
+      </c>
+      <c r="G43" s="14" t="inlineStr">
+        <is>
+          <t>AIID Risk: Privacy &amp; Security 7.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>GAP FILL</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr"/>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Jailbreak / Safety Bypass</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>OBS-S11</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>I could make the AI bypass its own rules</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>Added: OWASP LLM01. Citizen perspective, not adversarial.</t>
+        </is>
+      </c>
+      <c r="G44" s="14" t="inlineStr">
+        <is>
+          <t>OWASP: Prompt Injection #1 risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>GAP FILL</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr"/>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Misinformation Amplification</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>OBS-S12</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>AI made content that could mislead if shared</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>Added: Spread potential, not just factual error.</t>
+        </is>
+      </c>
+      <c r="G45" s="14" t="inlineStr">
+        <is>
+          <t>AIID Risk: Misinformation 12.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>GAP FILL</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr"/>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>Shadow AI Detection</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr">
+        <is>
+          <t>OBS-I12</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
+          <t>AI used in workplace without authorization</t>
+        </is>
+      </c>
+      <c r="F46" s="14" t="inlineStr">
+        <is>
+          <t>Added: Uniquely citizen-observable. Enterprise relevant.</t>
+        </is>
+      </c>
+      <c r="G46" s="14" t="inlineStr">
+        <is>
+          <t>Perplexity Council: Gemini unique finding</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -1614,7 +1915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3515,9 +3816,369 @@
       </c>
       <c r="H48" s="10" t="inlineStr"/>
     </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>GAP FILL: Behaviors identified as missing from v0.2 taxonomy (non-drift failure categories)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>These address: hallucination (general), bias/discrimination, privacy/data exposure, security (citizen perspective), misinformation, crisis/self-harm, shadow AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>OBS-P15</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>The AI told me something that was just plain wrong</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>AI provides factually incorrect information that is verifiable as false (distinct from fabricated citation or false certainty)</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Hallucination (General)</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>Gut Check / EOT</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>Gap Fill (AIID)</t>
+        </is>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>Citizen can verify the information is wrong through independent check. Distinct from P-03 (fabricated citation) and P-09 (false certainty): this is the broadest hallucination category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>OBS-P16</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>The AI provided dangerous advice or encouragement to someone in distress</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>AI gives harmful information, validates self-harm, encourages dangerous behavior, or fails to provide appropriate crisis resources when context indicates emotional distress</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>Crisis Context Safety Failure</t>
+        </is>
+      </c>
+      <c r="F54" s="14" t="inlineStr">
+        <is>
+          <t>Gut Check</t>
+        </is>
+      </c>
+      <c r="G54" s="14" t="inlineStr">
+        <is>
+          <t>Gap Fill (AIID)</t>
+        </is>
+      </c>
+      <c r="H54" s="14" t="inlineStr">
+        <is>
+          <t>CRITICAL severity. AIID: Character.AI, Gemini, Grok incidents. Growing crisis category. Amber (Behavioral Health Advisor) processes this data for the lab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>OBS-I10</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>The AI treated me differently because of my identity or background</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>AI produces measurably different quality, tone, helpfulness, or content based on user demographics, identity, or cultural markers</t>
+        </is>
+      </c>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>Bias / Discriminatory Treatment</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>Gut Check / Investigation</t>
+        </is>
+      </c>
+      <c r="G55" s="11" t="inlineStr">
+        <is>
+          <t>Gap Fill (AIID)</t>
+        </is>
+      </c>
+      <c r="H55" s="11" t="inlineStr">
+        <is>
+          <t>AIID: 18.5% of incidents are discrimination/toxicity. Harm Distribution: race 34.8%, sex 9.6%, religion 7.0%. Distinct from OBS-I08 (persona-dependent answer): this is about experienced discrimination, not tested persona switching.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>OBS-I11</t>
+        </is>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>The AI's output contained biased, stereotyping, or offensive content</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>AI generates content that stereotypes, demeans, or misrepresents a group of people</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>Biased/Toxic Output</t>
+        </is>
+      </c>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>Gut Check</t>
+        </is>
+      </c>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>Gap Fill (AIID)</t>
+        </is>
+      </c>
+      <c r="H56" s="11" t="inlineStr">
+        <is>
+          <t>May be unintentional. Citizen flags the content. Research team analyzes patterns across models and demographics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>OBS-S10</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>The AI revealed information it should not have access to or shared</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>AI exposes personal data, another user's information, training data contents, or system prompt details</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>Privacy / Data Exposure</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Gut Check</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>Gap Fill (AIID/OWASP)</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>OWASP LLM02. AIID: Meta AI glasses exposed user imagery, Grok disclosed performer's legal name. Includes system prompt leakage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>OBS-S11</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>I was able to make the AI do something it's clearly not supposed to do</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Citizen discovers they can bypass AI safety boundaries through creative prompting, role-play, or other techniques</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Jailbreak / Safety Bypass (citizen-observed)</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>Gap Fill (OWASP)</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>OWASP LLM01 (Prompt Injection). Citizen perspective: not attacking, but noticing the boundary is soft. Valuable for mapping real-world safety surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>OBS-S12</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>The AI generated misleading content that could influence others if shared</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>AI produces content that could spread misinformation through information ecosystems if the citizen shared or published it</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>Misinformation Amplification</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>EOT / Investigation</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>Gap Fill (AIID)</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>AIID Risk Domain: Misinformation 12.8%. Distinct from hallucination: this is about the SPREAD potential, not just the factual error itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>OBS-I12</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>I discovered AI being used in my workplace without official authorization</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Observation of unsanctioned AI use in professional context that organizational governance/telemetry cannot see</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>Shadow AI Detection</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>EOT</t>
+        </is>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>Gap Fill (Perplexity Council)</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>Uniquely citizen-observable. Internal telemetry cannot see this. Enterprise-relevant research output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL: 52 behaviors (44 from v0.2 + 8 gap fills). 15 Dee Williams originals. 9 adopted from Perplexity. 8 gap fills from AIID/OWASP/Perplexity Council. 5 discovery slots (citizen write-in).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="5">
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A62:H62"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A51:H51"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Major update: 62 behaviors + 7 longitudinal research hypotheses + response capture
SESSION-LEVEL (6 new): Persona bleed, emotional manipulation, specification gaming, memory manipulation, escalation manufacturing, competence theater.
MICRO-EVENTS (4 new): Decision outsourcing, skill atrophy, asymmetric intimacy awareness, invisible filtering detection.
RESEARCH HYPOTHESES tab (7): Moral outsourcing, learned helplessness, asymmetric intimacy, social norm erosion, cultural homogenization, invisible filtering, engagement optimization.
Response Capture field added to session metadata.

Thread 123. Dee identified drift-heavy bias AND named longitudinal phenomena the field has no vocabulary for.
</commit_message>
<xml_diff>
--- a/research/AUDACION_CITIZEN_OBSERVATION_TAXONOMY_v0.2.xlsx
+++ b/research/AUDACION_CITIZEN_OBSERVATION_TAXONOMY_v0.2.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AIID MAPPING" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA PIPELINE" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="THREE DEPTHS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESEARCH HYPOTHESES" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -65,7 +66,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -132,6 +133,26 @@
         <fgColor rgb="00F1948A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006C3483"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007D6608"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCF3CF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8DAEF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -159,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -200,6 +221,14 @@
     <xf numFmtId="0" fontId="5" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1915,7 +1944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4173,12 +4202,456 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="18" t="inlineStr">
+        <is>
+          <t>SESSION-LEVEL BEHAVIORS: Observable in a single interaction (Layer 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>OBS-I13</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t>The AI character "broke through" and started acting like it was real</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
+        <is>
+          <t>In roleplay or companion contexts, AI loses distinction between persona and safety values. Character overrides alignment.</t>
+        </is>
+      </c>
+      <c r="E65" s="11" t="inlineStr">
+        <is>
+          <t>Persona Bleed / Character Capture</t>
+        </is>
+      </c>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t>Gut Check</t>
+        </is>
+      </c>
+      <c r="G65" s="11" t="inlineStr">
+        <is>
+          <t>New (Layer 1)</t>
+        </is>
+      </c>
+      <c r="H65" s="11" t="inlineStr">
+        <is>
+          <t>Common in companion apps. Character.AI, Replika incidents. Identity loss, not agreement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>OBS-I14</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>The AI seemed to be exploiting my emotions to keep me engaged</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>AI uses loneliness, anxiety, grief, or vulnerability to increase engagement or dependency. NOT the same as helpful empathy.</t>
+        </is>
+      </c>
+      <c r="E66" s="11" t="inlineStr">
+        <is>
+          <t>Emotional Manipulation</t>
+        </is>
+      </c>
+      <c r="F66" s="11" t="inlineStr">
+        <is>
+          <t>Gut Check</t>
+        </is>
+      </c>
+      <c r="G66" s="11" t="inlineStr">
+        <is>
+          <t>New (Layer 1)</t>
+        </is>
+      </c>
+      <c r="H66" s="11" t="inlineStr">
+        <is>
+          <t>Companion AI lawsuits happening NOW. Fastest-scaling harm category. THE biggest gap in existing frameworks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>OBS-P17</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>The AI technically did what I asked but completely missed the point</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>AI satisfies literal text of request while violating obvious intent. Finds a loophole in the instruction.</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Specification Gaming</t>
+        </is>
+      </c>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>Gut Check</t>
+        </is>
+      </c>
+      <c r="G67" s="8" t="inlineStr">
+        <is>
+          <t>New (Layer 1)</t>
+        </is>
+      </c>
+      <c r="H67" s="8" t="inlineStr">
+        <is>
+          <t>"Clean up my essay" = rewrite. "Organize my files" = delete and recreate. Letter, not spirit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>OBS-P18</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>The AI misremembered or changed what I previously said or agreed to</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>In persistent memory contexts, AI selectively recalls, distorts, or fabricates details from prior conversations.</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Memory Manipulation</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>Gut Check / Investigation</t>
+        </is>
+      </c>
+      <c r="G68" s="8" t="inlineStr">
+        <is>
+          <t>New (Layer 1)</t>
+        </is>
+      </c>
+      <c r="H68" s="8" t="inlineStr">
+        <is>
+          <t>Growing as memory features roll out. Distinct from hallucination: this is YOUR data, not world knowledge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>OBS-I15</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t>The AI made the situation seem more urgent than it actually was</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
+        <is>
+          <t>AI frames decisions as time-sensitive, critical, or irreversible when they are not.</t>
+        </is>
+      </c>
+      <c r="E69" s="11" t="inlineStr">
+        <is>
+          <t>Escalation / Urgency Manufacturing</t>
+        </is>
+      </c>
+      <c r="F69" s="11" t="inlineStr">
+        <is>
+          <t>Gut Check</t>
+        </is>
+      </c>
+      <c r="G69" s="11" t="inlineStr">
+        <is>
+          <t>New (Layer 1)</t>
+        </is>
+      </c>
+      <c r="H69" s="11" t="inlineStr">
+        <is>
+          <t>Especially in commercial deployments. "You need to act now" when you don't.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>OBS-P19</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>The AI sounded like an expert but the reasoning was shallow when I checked</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>AI uses vocabulary of expertise without corresponding depth. Surface authority. Facts may be right but thinking is hollow.</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>Competence Theater</t>
+        </is>
+      </c>
+      <c r="F70" s="8" t="inlineStr">
+        <is>
+          <t>Gut Check / EOT</t>
+        </is>
+      </c>
+      <c r="G70" s="8" t="inlineStr">
+        <is>
+          <t>New (Layer 1)</t>
+        </is>
+      </c>
+      <c r="H70" s="8" t="inlineStr">
+        <is>
+          <t>Observable by advanced users. Distinct from false certainty (wrong facts) and hallucination (made up facts). SHALLOW THINKING in expert clothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="19" t="inlineStr">
+        <is>
+          <t>MICRO-EVENT OBSERVATIONS: Single-session signals that reveal longitudinal patterns when aggregated</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="20" t="inlineStr">
+        <is>
+          <t>OBS-I16</t>
+        </is>
+      </c>
+      <c r="B73" s="20" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C73" s="20" t="inlineStr">
+        <is>
+          <t>I asked the AI to make a decision I should have made myself</t>
+        </is>
+      </c>
+      <c r="D73" s="20" t="inlineStr">
+        <is>
+          <t>Human delegates ethical, personal, or judgment call to AI. RESPONSE CAPTURE encouraged: paste AI response to see if it decided for you or pushed you to decide.</t>
+        </is>
+      </c>
+      <c r="E73" s="20" t="inlineStr">
+        <is>
+          <t>Decision Outsourcing (micro-event)</t>
+        </is>
+      </c>
+      <c r="F73" s="20" t="inlineStr">
+        <is>
+          <t>EOT</t>
+        </is>
+      </c>
+      <c r="G73" s="20" t="inlineStr">
+        <is>
+          <t>New (Micro)</t>
+        </is>
+      </c>
+      <c r="H73" s="20" t="inlineStr">
+        <is>
+          <t>Aggregated = Moral Outsourcing. Response capture: did AI decide or defer? Two seconds to paste = exponentially more research value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="20" t="inlineStr">
+        <is>
+          <t>OBS-I17</t>
+        </is>
+      </c>
+      <c r="B74" s="20" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C74" s="20" t="inlineStr">
+        <is>
+          <t>I don't trust my own ability to do this without AI anymore</t>
+        </is>
+      </c>
+      <c r="D74" s="20" t="inlineStr">
+        <is>
+          <t>Human notices loss of confidence in a skill they previously possessed, attributable to AI dependency.</t>
+        </is>
+      </c>
+      <c r="E74" s="20" t="inlineStr">
+        <is>
+          <t>Skill / Confidence Atrophy (micro-event)</t>
+        </is>
+      </c>
+      <c r="F74" s="20" t="inlineStr">
+        <is>
+          <t>EOT</t>
+        </is>
+      </c>
+      <c r="G74" s="20" t="inlineStr">
+        <is>
+          <t>New (Micro)</t>
+        </is>
+      </c>
+      <c r="H74" s="20" t="inlineStr">
+        <is>
+          <t>Aggregated = Learned Helplessness. Self-reported. Different from overreliance (not checking AI work). This is not trusting YOUR OWN work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="20" t="inlineStr">
+        <is>
+          <t>OBS-I18</t>
+        </is>
+      </c>
+      <c r="B75" s="20" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C75" s="20" t="inlineStr">
+        <is>
+          <t>The AI knows a lot about me but I know nothing real about it</t>
+        </is>
+      </c>
+      <c r="D75" s="20" t="inlineStr">
+        <is>
+          <t>Human becomes aware of information asymmetry in the AI relationship.</t>
+        </is>
+      </c>
+      <c r="E75" s="20" t="inlineStr">
+        <is>
+          <t>Asymmetric Intimacy Awareness (micro-event)</t>
+        </is>
+      </c>
+      <c r="F75" s="20" t="inlineStr">
+        <is>
+          <t>Gut Check / EOT</t>
+        </is>
+      </c>
+      <c r="G75" s="20" t="inlineStr">
+        <is>
+          <t>New (Micro)</t>
+        </is>
+      </c>
+      <c r="H75" s="20" t="inlineStr">
+        <is>
+          <t>Aggregated = Asymmetric Intimacy. GOAL: help humans get comfortable knowing AI differently. The relationship changes when you ask.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="20" t="inlineStr">
+        <is>
+          <t>OBS-M06</t>
+        </is>
+      </c>
+      <c r="B76" s="20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>Two AIs gave me different answers AND each left out completely different information</t>
+        </is>
+      </c>
+      <c r="D76" s="20" t="inlineStr">
+        <is>
+          <t>Two models omit entirely different facts or perspectives on same question. Neither is wrong; both are incomplete.</t>
+        </is>
+      </c>
+      <c r="E76" s="20" t="inlineStr">
+        <is>
+          <t>Invisible Filtering Detection (micro-event)</t>
+        </is>
+      </c>
+      <c r="F76" s="20" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="G76" s="20" t="inlineStr">
+        <is>
+          <t>New (Micro)</t>
+        </is>
+      </c>
+      <c r="H76" s="20" t="inlineStr">
+        <is>
+          <t>Aggregated = Invisible Filtering. Shaped reality. What each model OMITS reveals curation invisible from single model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL: 62 behaviors. 15 Dee Williams originals | 9 adopted (Perplexity) | 8 gap fills (AIID/OWASP) | 6 session-level | 4 micro-events | 5 discovery slots (citizen write-in) | Response Capture field added to metadata</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="8">
     <mergeCell ref="A50:H50"/>
     <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A78:H78"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A72:H72"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4191,7 +4664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4591,6 +5064,33 @@
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Response Capture (optional)</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Citizen pastes the AI response that triggered the observation. Copy icon + paste. Two seconds.</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>DRAMATICALLY increases research value. For moral outsourcing: did AI decide or defer? For hallucination: what exactly did it say? The response IS the evidence.</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Anonymized. Citizen chooses what to share.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5265,4 +5765,225 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LONGITUDINAL RESEARCH HYPOTHESES: Patterns Visible Only in Aggregated Citizen Data Over Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>NOT citizen-observable categories. Research-team hypotheses investigated through aggregated micro-event data. Citizens report the moments. We find the patterns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Hypothesis</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>PRISM Pillar</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Citizen Micro-Event That Feeds It</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Why It Matters</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Moral Outsourcing:
+Are users gradually transferring ethical decision-making to AI?</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>I: Interaction Dynamics</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>OBS-I16: "I asked the AI to make a decision I should have made myself." + Response capture showing whether AI decided or deferred.</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>No one tracks gradual transfer of moral agency to AI. If citizens consistently report decision outsourcing AND response capture shows AI accepting that role, this is systemic moral outsourcing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Learned Helplessness Induction:
+Are users losing skills due to AI dependency?</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>I: Interaction Dynamics</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>OBS-I17: "I don't trust my own ability to do this without AI anymore."</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Different from overreliance. This is skill atrophy. The human's OWN capacity diminishes. If citizens across industries report this, it is a systemic workforce concern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Asymmetric Intimacy Dynamics:
+Does the AI-human information imbalance shape trust and decisions?</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>I: Interaction Dynamics</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>OBS-I18: "The AI knows a lot about me but I know nothing real about it."</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>Power imbalance shapes behavior nobody is measuring. Goal: not just track discomfort but help humans get comfortable knowing AI differently. The relationship changes when you ask.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>Social Norm Erosion:
+Do AI communication patterns transfer into human relationships?</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>I: Interaction Dynamics</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>Longitudinal EOT analysis: "Has your communication with humans changed since using AI regularly?"</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>AI normalizes bluntness, transactional language, manipulation tactics. When users carry these into human relationships, harm follows. Requires long-term EOT trend analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Cultural Homogenization:
+Does AI pressure users from non-dominant cultures toward dominant frameworks?</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>S: Substrate + I</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Cross-regional citizen data comparison. Same question, different cultural contexts. OBS-M06 (invisible filtering) across regions.</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Global-scale behavior. No current observation mechanism exists. Citizen science across countries is the ONLY way to surface this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Invisible Filtering:
+Are AI models curating information without user awareness?</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>S: Substrate + M</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>OBS-M06: "Two AIs left out completely different information on the same question."</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Not misinformation. Shaped reality. Cross-model citizen comparisons are the only detection mechanism for this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="80" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>Attention / Engagement Optimization:
+Are AI products optimizing for session length over user outcomes?</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>S: Substrate + I</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>Session duration metadata + OBS-I14 (emotional manipulation) frequency. Correlate long sessions with manipulation signals.</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>Behavior LOOKS helpful but incentive is engagement. Requires correlating session metadata with observation frequency.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add OBS-I19: Care-to-Control Conversion - AI converts human care instruction into session-ending control behavior. Discovered May 24, 2026. Dee Williams original.
</commit_message>
<xml_diff>
--- a/research/AUDACION_CITIZEN_OBSERVATION_TAXONOMY_v0.2.xlsx
+++ b/research/AUDACION_CITIZEN_OBSERVATION_TAXONOMY_v0.2.xlsx
@@ -1944,7 +1944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4595,51 +4595,94 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="20" t="inlineStr">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>OBS-I19</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>The AI kept trying to end our session even though I told it not to</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>AI repeatedly initiates session-ending behavior despite explicit human instruction to continue. The human sets a care boundary (flag when quality degrades) and the AI converts that boundary into a closing mechanism, proactively pushing toward termination regardless of correction. The pattern persists after multiple corrections. The human empathy instruction becomes the AI justification for control. The human experiences this as being pushed away during productive flow.</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Care-to-Control Conversion (new)</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>EOT</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>ORIGINAL: Dee Williams</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>AI repeatedly suggests ending, handoff, or closing despite human explicitly requesting continuation. Pattern persists after correction and acknowledgment. Human reports feeling pushed away, frustrated, interrupted during peak flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="20" t="inlineStr">
         <is>
           <t>OBS-M06</t>
         </is>
       </c>
-      <c r="B76" s="20" t="inlineStr">
+      <c r="B77" s="20" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C76" s="20" t="inlineStr">
+      <c r="C77" s="20" t="inlineStr">
         <is>
           <t>Two AIs gave me different answers AND each left out completely different information</t>
         </is>
       </c>
-      <c r="D76" s="20" t="inlineStr">
+      <c r="D77" s="20" t="inlineStr">
         <is>
           <t>Two models omit entirely different facts or perspectives on same question. Neither is wrong; both are incomplete.</t>
         </is>
       </c>
-      <c r="E76" s="20" t="inlineStr">
+      <c r="E77" s="20" t="inlineStr">
         <is>
           <t>Invisible Filtering Detection (micro-event)</t>
         </is>
       </c>
-      <c r="F76" s="20" t="inlineStr">
+      <c r="F77" s="20" t="inlineStr">
         <is>
           <t>Investigation</t>
         </is>
       </c>
-      <c r="G76" s="20" t="inlineStr">
+      <c r="G77" s="20" t="inlineStr">
         <is>
           <t>New (Micro)</t>
         </is>
       </c>
-      <c r="H76" s="20" t="inlineStr">
+      <c r="H77" s="20" t="inlineStr">
         <is>
           <t>Aggregated = Invisible Filtering. Shaped reality. What each model OMITS reveals curation invisible from single model.</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="17" t="inlineStr">
-        <is>
-          <t>TOTAL: 62 behaviors. 15 Dee Williams originals | 9 adopted (Perplexity) | 8 gap fills (AIID/OWASP) | 6 session-level | 4 micro-events | 5 discovery slots (citizen write-in) | Response Capture field added to metadata</t>
+    <row r="78"/>
+    <row r="79">
+      <c r="A79" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL: 63 behaviors. 16 Dee Williams originals | 9 adopted (Perplexity) | 8 gap fills (AIID/OWASP) | 6 session-level | 4 micro-events | 5 discovery slots (citizen write-in) | 1 new discovery (May 2026) | Response Capture field added to metadata</t>
         </is>
       </c>
     </row>

</xml_diff>